<commit_message>
update no coupling condition
</commit_message>
<xml_diff>
--- a/simulated_data/dyads_simulated/cond3_no_coupling/HRV_A.xlsx
+++ b/simulated_data/dyads_simulated/cond3_no_coupling/HRV_A.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A543"/>
+  <dimension ref="A1:A541"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -430,2707 +430,2697 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>474</v>
+        <v>761.4487978993438</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>766</v>
+        <v>824.8288076933743</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>752</v>
+        <v>848.8670358156387</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>674</v>
+        <v>889.1076968391465</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>640</v>
+        <v>860.6775662917903</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>628</v>
+        <v>888.7171874020563</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>644</v>
+        <v>948.0659674185858</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>730</v>
+        <v>894.1219748432729</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>800</v>
+        <v>851.3458723861688</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>854</v>
+        <v>825.6939708287732</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>854</v>
+        <v>890.3364728603531</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>838</v>
+        <v>921.5916376395619</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>814</v>
+        <v>775.0149108295652</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>766</v>
+        <v>795.930069386877</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>736</v>
+        <v>778.7595938768721</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>670</v>
+        <v>718.5163272214456</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>640</v>
+        <v>774.9288923946835</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>630</v>
+        <v>725.6484797602862</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>612</v>
+        <v>752.2517117957434</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>610</v>
+        <v>882.4074588108103</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>674</v>
+        <v>886.3631571264427</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>754</v>
+        <v>854.8455345804698</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>832</v>
+        <v>822.7514611785195</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>840</v>
+        <v>839.0705213178684</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>786</v>
+        <v>819.3817456566244</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>800</v>
+        <v>788.9524542250897</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>822</v>
+        <v>860.5817754434781</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>804</v>
+        <v>839.7500542402056</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>814</v>
+        <v>883.2412077990597</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>838</v>
+        <v>873.9752872771902</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>844</v>
+        <v>831.2274263076382</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>846</v>
+        <v>737.5643264669698</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>830</v>
+        <v>790.0824858066393</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>816</v>
+        <v>910.5026867996422</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>740</v>
+        <v>929.1931125080772</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>712</v>
+        <v>874.0591075634221</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>750</v>
+        <v>876.9568415265461</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>818</v>
+        <v>820.0032832504434</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>778</v>
+        <v>825.7256288945847</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>716</v>
+        <v>801.204369014549</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>816</v>
+        <v>797.7189128631323</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>756</v>
+        <v>858.3693120655198</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>726</v>
+        <v>853.3165754496893</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>768</v>
+        <v>824.570153306702</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>828</v>
+        <v>820.2618749445846</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>920</v>
+        <v>832.7480797248584</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>956</v>
+        <v>855.3668509267354</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>868</v>
+        <v>901.5982145621422</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>872</v>
+        <v>869.3947412036707</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>886</v>
+        <v>788.944149877615</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>880</v>
+        <v>720.5461628034514</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>796</v>
+        <v>756.9026919864327</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>820</v>
+        <v>843.211532261229</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>804</v>
+        <v>945.8446367934386</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>836</v>
+        <v>908.5253615575795</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>876</v>
+        <v>895.7402219963058</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>956</v>
+        <v>809.5368402795486</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>948</v>
+        <v>744.0190230415595</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>916</v>
+        <v>718.3028423130154</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>900</v>
+        <v>770.5716644644056</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>854</v>
+        <v>796.5580401500531</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>794</v>
+        <v>837.2071332596107</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>704</v>
+        <v>908.5415826390175</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>682</v>
+        <v>859.3231647953062</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>708</v>
+        <v>777.8453622536148</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>706</v>
+        <v>722.506880726037</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>712</v>
+        <v>741.8443953483163</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>970</v>
+        <v>791.4911569596015</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>986</v>
+        <v>866.6846841348672</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>948</v>
+        <v>974.4957224452762</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>982</v>
+        <v>959.2115047884135</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>980</v>
+        <v>853.8944591727429</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>882</v>
+        <v>799.4801028580341</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>842</v>
+        <v>849.5577206678249</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>942</v>
+        <v>888.9544364092999</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>994</v>
+        <v>957.6413644973769</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>936</v>
+        <v>907.9682104791473</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>846</v>
+        <v>918.8222503857162</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>866</v>
+        <v>843.954284154151</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>918</v>
+        <v>838.468138600561</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>900</v>
+        <v>881.9963097936778</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>826</v>
+        <v>755.6272931373513</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>876</v>
+        <v>772.773754188421</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>930</v>
+        <v>712.1749871797363</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>930</v>
+        <v>710.6863974088782</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>846</v>
+        <v>790.8284374185968</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>856</v>
+        <v>853.7851196118424</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>894</v>
+        <v>848.0859990340548</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>916</v>
+        <v>842.4251527607964</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>850</v>
+        <v>833.2345938772505</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>810</v>
+        <v>744.8568583483706</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>870</v>
+        <v>726.0737731112528</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>934</v>
+        <v>692.7363065976095</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>916</v>
+        <v>726.1293477600219</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>824</v>
+        <v>759.3519871424803</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>826</v>
+        <v>783.2620603507507</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>780</v>
+        <v>829.1090296636838</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>702</v>
+        <v>857.5197253963012</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>720</v>
+        <v>834.8362787294832</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>856</v>
+        <v>720.6140477843661</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>872</v>
+        <v>688.5724049077737</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>902</v>
+        <v>707.9833864781904</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>904</v>
+        <v>758.6518322114557</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>772</v>
+        <v>819.9402096799702</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>700</v>
+        <v>887.517885843252</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>668</v>
+        <v>945.9113111865491</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>668</v>
+        <v>908.3670799210353</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>688</v>
+        <v>829.7357678151798</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>726</v>
+        <v>700.7896622013163</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>762</v>
+        <v>657.9976697387764</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>818</v>
+        <v>724.0059926773341</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>840</v>
+        <v>820.1955116534663</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>852</v>
+        <v>808.2128209250499</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>846</v>
+        <v>769.6216591834286</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>812</v>
+        <v>805.6410894362642</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>766</v>
+        <v>882.8020614252523</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>732</v>
+        <v>925.6240124038584</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>714</v>
+        <v>922.5902970039641</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>692</v>
+        <v>863.6246392143505</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>670</v>
+        <v>737.332905546765</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>664</v>
+        <v>693.5861477301444</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>662</v>
+        <v>739.3431688923044</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>670</v>
+        <v>756.9323038182318</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>692</v>
+        <v>813.7567813813149</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>696</v>
+        <v>866.3548169218558</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>674</v>
+        <v>876.193299030092</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>692</v>
+        <v>812.2007431643823</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>774</v>
+        <v>744.7363356646832</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>756</v>
+        <v>719.7275583622087</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>816</v>
+        <v>755.3520735013279</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>838</v>
+        <v>725.3791535504206</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>818</v>
+        <v>710.4626203647797</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>784</v>
+        <v>846.4996425706346</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>690</v>
+        <v>989.9999999999949</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>640</v>
+        <v>989.9999999999949</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>632</v>
+        <v>892.5457707599662</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>694</v>
+        <v>803.5703777918854</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>834</v>
+        <v>797.6656564046749</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>896</v>
+        <v>817.7690370037851</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>924</v>
+        <v>870.3600451538449</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>886</v>
+        <v>863.0041365651664</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>790</v>
+        <v>825.6741433013275</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>710</v>
+        <v>775.8352546368599</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>746</v>
+        <v>838.0535468280641</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>778</v>
+        <v>887.5892060064388</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>788</v>
+        <v>900.7212942330796</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>802</v>
+        <v>900.402321286478</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>812</v>
+        <v>821.4858759414767</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>792</v>
+        <v>823.0016108553997</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>724</v>
+        <v>803.5869757524239</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>676</v>
+        <v>723.8766777797991</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>660</v>
+        <v>670.5665049105107</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>660</v>
+        <v>680.9317456918791</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>650</v>
+        <v>694.2618598728103</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>680</v>
+        <v>770.6668632888238</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>744</v>
+        <v>846.1184386663376</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>772</v>
+        <v>804.217223215403</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>776</v>
+        <v>789.2267515758817</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>828</v>
+        <v>747.4502110023877</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>864</v>
+        <v>734.9545268874067</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>776</v>
+        <v>749.7610658409997</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
-        <v>784</v>
+        <v>756.1088286984727</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
-        <v>800</v>
+        <v>688.877530063138</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
-        <v>828</v>
+        <v>678.9513930841338</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>840</v>
+        <v>773.0974770217642</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
-        <v>818</v>
+        <v>848.3594131463121</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
-        <v>808</v>
+        <v>836.4110793971236</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
-        <v>810</v>
+        <v>845.8481127616722</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
-        <v>796</v>
+        <v>764.9795533608028</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
-        <v>802</v>
+        <v>681.5679913939334</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
-        <v>778</v>
+        <v>627.7755711319628</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
-        <v>712</v>
+        <v>671.6491630703558</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
-        <v>674</v>
+        <v>718.6250553222351</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
-        <v>672</v>
+        <v>781.8268582448411</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
-        <v>738</v>
+        <v>776.6267508255851</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>864</v>
+        <v>809.7783523604107</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>880</v>
+        <v>855.9025085079099</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>776</v>
+        <v>837.9976952383288</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>752</v>
+        <v>820.3356190259967</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>724</v>
+        <v>787.0725013997912</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>682</v>
+        <v>800.9066671104961</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>754</v>
+        <v>746.3271046757995</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>874</v>
+        <v>705.1819953960319</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>820</v>
+        <v>731.5393981065483</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>836</v>
+        <v>794.2336162363688</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>750</v>
+        <v>832.1230316527988</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>754</v>
+        <v>860.7340775477326</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>782</v>
+        <v>837.4853100571613</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>856</v>
+        <v>802.0609306539654</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>914</v>
+        <v>810.1082430666509</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>932</v>
+        <v>784.5641019264065</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>892</v>
+        <v>877.2285667557469</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>836</v>
+        <v>973.274249412583</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
-        <v>792</v>
+        <v>990.0000000000091</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
-        <v>730</v>
+        <v>980.6026046300076</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
-        <v>690</v>
+        <v>861.9492009626128</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
-        <v>690</v>
+        <v>792.8109865585498</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
-        <v>802</v>
+        <v>793.9141248838553</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
-        <v>924</v>
+        <v>781.2427016936851</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>860</v>
+        <v>845.6265241151186</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
-        <v>870</v>
+        <v>917.3570624905665</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
-        <v>878</v>
+        <v>834.3198328943799</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="n">
-        <v>876</v>
+        <v>868.5333742043895</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
-        <v>870</v>
+        <v>878.3665293049125</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
-        <v>856</v>
+        <v>925.6598101086411</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="n">
-        <v>730</v>
+        <v>951.4156376945095</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="n">
-        <v>684</v>
+        <v>899.8215196984063</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="n">
-        <v>642</v>
+        <v>934.3076125098264</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="n">
-        <v>656</v>
+        <v>951.6825810605667</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="n">
-        <v>844</v>
+        <v>888.8183417919322</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="n">
-        <v>912</v>
+        <v>884.6984207423532</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="n">
-        <v>932</v>
+        <v>921.1887113625323</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="n">
-        <v>934</v>
+        <v>902.1943746096213</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="n">
-        <v>908</v>
+        <v>862.1201212541223</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="n">
-        <v>800</v>
+        <v>844.9192824428735</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="n">
-        <v>824</v>
+        <v>805.4191136324391</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="n">
-        <v>898</v>
+        <v>893.2455614376238</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="n">
-        <v>938</v>
+        <v>953.0032349981923</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="n">
-        <v>944</v>
+        <v>989.6413086252096</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="n">
-        <v>866</v>
+        <v>990.0000000000091</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="n">
-        <v>782</v>
+        <v>990.0000000000091</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="n">
-        <v>816</v>
+        <v>953.2948452317385</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="n">
-        <v>836</v>
+        <v>945.5144577658814</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="n">
-        <v>862</v>
+        <v>859.5802660915979</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="n">
-        <v>776</v>
+        <v>900.6712508740407</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="n">
-        <v>820</v>
+        <v>858.1070112391274</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="n">
-        <v>842</v>
+        <v>812.761788291823</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="n">
-        <v>902</v>
+        <v>829.3701501514761</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="n">
-        <v>922</v>
+        <v>841.5526653750192</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="n">
-        <v>876</v>
+        <v>829.5838562612232</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="n">
-        <v>790</v>
+        <v>837.2107383261209</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="n">
-        <v>800</v>
+        <v>900.2020390787777</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="n">
-        <v>812</v>
+        <v>930.2685066670335</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="n">
-        <v>844</v>
+        <v>883.2097704776345</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="n">
-        <v>860</v>
+        <v>897.2836690547297</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="n">
-        <v>756</v>
+        <v>925.1302630758289</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="n">
-        <v>702</v>
+        <v>912.9915198112997</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="n">
-        <v>720</v>
+        <v>840.7953317412478</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="n">
-        <v>726</v>
+        <v>810.2868181876204</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="n">
-        <v>704</v>
+        <v>801.6506830775825</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="n">
-        <v>668</v>
+        <v>806.6729214608301</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="n">
-        <v>676</v>
+        <v>817.0745984210441</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="n">
-        <v>724</v>
+        <v>838.5894945731138</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="n">
-        <v>750</v>
+        <v>876.0665988450569</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="n">
-        <v>700</v>
+        <v>867.7281796707916</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="n">
-        <v>712</v>
+        <v>960.1941948793353</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="n">
-        <v>746</v>
+        <v>964.625192483652</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="n">
-        <v>798</v>
+        <v>937.3027574568766</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="n">
-        <v>756</v>
+        <v>893.9512843639648</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="n">
-        <v>804</v>
+        <v>904.7719309160698</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="n">
-        <v>864</v>
+        <v>816.8056567103577</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="n">
-        <v>898</v>
+        <v>763.7288123405312</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="n">
-        <v>890</v>
+        <v>782.7163261032126</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="n">
-        <v>816</v>
+        <v>790.6983901037847</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="n">
-        <v>746</v>
+        <v>888.9700265056888</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="n">
-        <v>744</v>
+        <v>960.0214218619953</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="n">
-        <v>776</v>
+        <v>950.4267997035072</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="n">
-        <v>852</v>
+        <v>896.9275353905459</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="n">
-        <v>910</v>
+        <v>826.8969149004022</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="n">
-        <v>838</v>
+        <v>813.945064858018</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="n">
-        <v>818</v>
+        <v>831.7800899345968</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="n">
-        <v>880</v>
+        <v>868.1028922399605</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="n">
-        <v>926</v>
+        <v>924.2099591399722</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="n">
-        <v>864</v>
+        <v>865.9850837966303</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="n">
-        <v>780</v>
+        <v>817.9167897746424</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="n">
-        <v>786</v>
+        <v>869.9286022990975</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="n">
-        <v>808</v>
+        <v>825.9345863640988</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="n">
-        <v>790</v>
+        <v>800.1859460642606</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="n">
-        <v>840</v>
+        <v>741.8573443118532</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="n">
-        <v>860</v>
+        <v>837.6092589077189</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="n">
-        <v>858</v>
+        <v>947.1137608426545</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="n">
-        <v>846</v>
+        <v>883.4028991703917</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="n">
-        <v>754</v>
+        <v>857.768160979731</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="n">
-        <v>710</v>
+        <v>822.1954869115393</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="n">
-        <v>666</v>
+        <v>786.8187491135075</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="n">
-        <v>724</v>
+        <v>816.6135228151745</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="n">
-        <v>804</v>
+        <v>736.3917140089029</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="n">
-        <v>898</v>
+        <v>662.509827036331</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="n">
-        <v>940</v>
+        <v>671.638259429244</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="n">
-        <v>922</v>
+        <v>744.9170014887727</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="n">
-        <v>904</v>
+        <v>811.0888191787922</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="n">
-        <v>806</v>
+        <v>812.0165243618089</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="n">
-        <v>758</v>
+        <v>829.2347115677217</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="n">
-        <v>724</v>
+        <v>780.1091136061871</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="n">
-        <v>736</v>
+        <v>703.9486697624113</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="n">
-        <v>742</v>
+        <v>646.5753496811146</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="n">
-        <v>768</v>
+        <v>642.4446599568796</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="n">
-        <v>850</v>
+        <v>665.4843177516341</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="n">
-        <v>930</v>
+        <v>698.9739460886994</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="n">
-        <v>938</v>
+        <v>757.4705879304418</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="n">
-        <v>802</v>
+        <v>859.0356853355843</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="n">
-        <v>768</v>
+        <v>889.0758847313123</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="n">
-        <v>772</v>
+        <v>861.9176254008494</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="n">
-        <v>750</v>
+        <v>843.8283351491691</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="n">
-        <v>820</v>
+        <v>843.3964898663646</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="n">
-        <v>866</v>
+        <v>768.3797902552953</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="n">
-        <v>876</v>
+        <v>725.3939004042138</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="n">
-        <v>876</v>
+        <v>700.4405733777048</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="n">
-        <v>828</v>
+        <v>781.5717978209022</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="n">
-        <v>750</v>
+        <v>867.6412766676265</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="n">
-        <v>752</v>
+        <v>864.970936912357</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="n">
-        <v>794</v>
+        <v>788.1503745419138</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="n">
-        <v>786</v>
+        <v>775.4089630231817</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="n">
-        <v>838</v>
+        <v>702.3965917812518</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="n">
-        <v>784</v>
+        <v>791.2380398742584</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="n">
-        <v>848</v>
+        <v>849.8998214394078</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="n">
-        <v>894</v>
+        <v>889.4241374852925</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="n">
-        <v>902</v>
+        <v>923.5743223894985</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="n">
-        <v>872</v>
+        <v>943.537707293018</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="n">
-        <v>754</v>
+        <v>819.7389713136261</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="n">
-        <v>706</v>
+        <v>761.7731212812373</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="n">
-        <v>704</v>
+        <v>759.0712291789146</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="n">
-        <v>750</v>
+        <v>822.7402383868139</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="n">
-        <v>792</v>
+        <v>853.9109012747303</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="n">
-        <v>792</v>
+        <v>881.6192492936352</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="n">
-        <v>816</v>
+        <v>972.8556598817022</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="n">
-        <v>806</v>
+        <v>989.9755443753406</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="n">
-        <v>784</v>
+        <v>966.3539481234125</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="n">
-        <v>766</v>
+        <v>970.6628129285946</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="n">
-        <v>752</v>
+        <v>913.8683148156588</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="n">
-        <v>694</v>
+        <v>782.0856696764622</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="n">
-        <v>668</v>
+        <v>722.7392628792018</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="n">
-        <v>654</v>
+        <v>755.8003563369198</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="n">
-        <v>648</v>
+        <v>794.5263306809807</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="n">
-        <v>762</v>
+        <v>810.1981963635581</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="n">
-        <v>882</v>
+        <v>814.0266616089207</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="n">
-        <v>978</v>
+        <v>843.0506681692691</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="n">
-        <v>990</v>
+        <v>897.3080193527494</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="n">
-        <v>932</v>
+        <v>983.6506047210491</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="n">
-        <v>872</v>
+        <v>981.4715165150005</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="n">
-        <v>872</v>
+        <v>921.4249046950727</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="n">
-        <v>816</v>
+        <v>834.8475074823796</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="n">
-        <v>840</v>
+        <v>816.9159097481611</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="n">
-        <v>858</v>
+        <v>908.1335850427195</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="n">
-        <v>872</v>
+        <v>956.0122260343178</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="n">
-        <v>898</v>
+        <v>990.0000000000091</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="n">
-        <v>928</v>
+        <v>905.1768337482144</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="n">
-        <v>870</v>
+        <v>928.4869521324026</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="n">
-        <v>888</v>
+        <v>911.9575893457181</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="n">
-        <v>888</v>
+        <v>854.9186097129109</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="n">
-        <v>882</v>
+        <v>861.7014613089964</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="n">
-        <v>902</v>
+        <v>874.7622403683408</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="n">
-        <v>914</v>
+        <v>849.2093388968556</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="n">
-        <v>892</v>
+        <v>799.5988088433705</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="n">
-        <v>878</v>
+        <v>735.0021000755191</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="n">
-        <v>796</v>
+        <v>777.7746679669235</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="n">
-        <v>772</v>
+        <v>853.7300781037516</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="n">
-        <v>766</v>
+        <v>881.7855775677117</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="n">
-        <v>756</v>
+        <v>875.8756075213228</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="n">
-        <v>772</v>
+        <v>901.9368182924268</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="n">
-        <v>810</v>
+        <v>970.7144285989102</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="n">
-        <v>854</v>
+        <v>944.2536172193172</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="n">
-        <v>854</v>
+        <v>850.0435155601167</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="n">
-        <v>852</v>
+        <v>772.1883074849529</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="n">
-        <v>832</v>
+        <v>772.1411169493422</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="n">
-        <v>790</v>
+        <v>734.7435412899017</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="n">
-        <v>776</v>
+        <v>764.5914053702541</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="n">
-        <v>754</v>
+        <v>819.8193038057866</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="n">
-        <v>756</v>
+        <v>815.4159720838834</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="n">
-        <v>726</v>
+        <v>838.6874026650162</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="n">
-        <v>788</v>
+        <v>906.4517856911607</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="n">
-        <v>856</v>
+        <v>972.5104279893344</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="n">
-        <v>916</v>
+        <v>920.8446360491394</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="n">
-        <v>936</v>
+        <v>831.4789065540253</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="n">
-        <v>900</v>
+        <v>784.0092718267329</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="n">
-        <v>848</v>
+        <v>831.3016822939971</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="n">
-        <v>814</v>
+        <v>814.7054249838561</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="n">
-        <v>752</v>
+        <v>760.8602114011092</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="n">
-        <v>704</v>
+        <v>762.767049583374</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="n">
-        <v>700</v>
+        <v>794.8545105600715</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="n">
-        <v>796</v>
+        <v>823.4059429400418</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="n">
-        <v>868</v>
+        <v>856.9578157342903</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="n">
-        <v>910</v>
+        <v>855.54846434502</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="n">
-        <v>906</v>
+        <v>824.3892482080923</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="n">
-        <v>844</v>
+        <v>815.850922056427</v>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="n">
-        <v>840</v>
+        <v>801.9525474037437</v>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="n">
-        <v>868</v>
+        <v>824.430743643461</v>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="n">
-        <v>768</v>
+        <v>858.7520627098115</v>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="n">
-        <v>692</v>
+        <v>865.6584856354925</v>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="n">
-        <v>752</v>
+        <v>868.6045286165722</v>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="n">
-        <v>854</v>
+        <v>898.4600704692411</v>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="n">
-        <v>920</v>
+        <v>806.1606106206227</v>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="n">
-        <v>942</v>
+        <v>716.9796491715488</v>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="n">
-        <v>880</v>
+        <v>776.0873632829544</v>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="n">
-        <v>790</v>
+        <v>851.1863291566897</v>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="n">
-        <v>728</v>
+        <v>833.7284658645672</v>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="n">
-        <v>704</v>
+        <v>751.7283914111204</v>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="n">
-        <v>892</v>
+        <v>802.0982626831028</v>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="n">
-        <v>900</v>
+        <v>847.5477319202582</v>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="n">
-        <v>972</v>
+        <v>797.1710487279893</v>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="n">
-        <v>890</v>
+        <v>777.03170420898</v>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="n">
-        <v>910</v>
+        <v>814.8910729779573</v>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="n">
-        <v>936</v>
+        <v>828.4796323567889</v>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="n">
-        <v>860</v>
+        <v>790.1987704455564</v>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="n">
-        <v>882</v>
+        <v>738.9194755402286</v>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="n">
-        <v>924</v>
+        <v>778.6110299837219</v>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="n">
-        <v>988</v>
+        <v>876.3570757423054</v>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="n">
-        <v>960</v>
+        <v>853.0276436850954</v>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="n">
-        <v>852</v>
+        <v>814.2497771829085</v>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="n">
-        <v>864</v>
+        <v>787.0174789980524</v>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="n">
-        <v>890</v>
+        <v>755.9241267271091</v>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="n">
-        <v>922</v>
+        <v>669.6613067604176</v>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="n">
-        <v>968</v>
+        <v>718.0984110266877</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="n">
-        <v>880</v>
+        <v>801.7090817771191</v>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="n">
-        <v>810</v>
+        <v>823.6265462630286</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="n">
-        <v>854</v>
+        <v>875.5631189340534</v>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="n">
-        <v>956</v>
+        <v>911.1031254479371</v>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="n">
-        <v>928</v>
+        <v>842.9307008158275</v>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="n">
-        <v>906</v>
+        <v>635.1771861998827</v>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="n">
-        <v>908</v>
+        <v>541.9321277856284</v>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="n">
-        <v>912</v>
+        <v>540.9149001172864</v>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="n">
-        <v>808</v>
+        <v>583.5742043900609</v>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="n">
-        <v>842</v>
+        <v>646.5650836384498</v>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="n">
-        <v>840</v>
+        <v>771.2499403062338</v>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="n">
-        <v>860</v>
+        <v>819.0850420155584</v>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="n">
-        <v>782</v>
+        <v>788.5072762649088</v>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="n">
-        <v>766</v>
+        <v>819.2039658911199</v>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="n">
-        <v>778</v>
+        <v>829.0856122105197</v>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="n">
-        <v>852</v>
+        <v>842.6834376560919</v>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="n">
-        <v>828</v>
+        <v>841.6435514024556</v>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="n">
-        <v>888</v>
+        <v>922.4566964380756</v>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="n">
-        <v>928</v>
+        <v>883.1162894114186</v>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="n">
-        <v>926</v>
+        <v>773.6058810943973</v>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="n">
-        <v>914</v>
+        <v>733.2098954923367</v>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="n">
-        <v>838</v>
+        <v>799.6058254723266</v>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="n">
-        <v>788</v>
+        <v>879.8987354924748</v>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="n">
-        <v>738</v>
+        <v>892.6518488004263</v>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="n">
-        <v>738</v>
+        <v>960.2949688812146</v>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="n">
-        <v>792</v>
+        <v>863.1350054341169</v>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="n">
-        <v>894</v>
+        <v>785.5119362754976</v>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="n">
-        <v>818</v>
+        <v>719.1482468870731</v>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="n">
-        <v>796</v>
+        <v>705.9151053602477</v>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="n">
-        <v>904</v>
+        <v>714.6401982827797</v>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="n">
-        <v>940</v>
+        <v>799.755104797498</v>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="n">
-        <v>878</v>
+        <v>871.6331180268639</v>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="n">
-        <v>878</v>
+        <v>934.586058338482</v>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="n">
-        <v>860</v>
+        <v>852.7033343823405</v>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="n">
-        <v>786</v>
+        <v>822.2585947144694</v>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="n">
-        <v>810</v>
+        <v>778.6718168991911</v>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="n">
-        <v>834</v>
+        <v>771.8138732136026</v>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="n">
-        <v>866</v>
+        <v>750.3861080770093</v>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="n">
-        <v>866</v>
+        <v>751.7395643300802</v>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="n">
-        <v>812</v>
+        <v>796.4878325978475</v>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="n">
-        <v>802</v>
+        <v>790.1267798874869</v>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="n">
-        <v>818</v>
+        <v>840.4511443399656</v>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="n">
-        <v>830</v>
+        <v>834.8655159701366</v>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="n">
-        <v>830</v>
+        <v>894.5966714592259</v>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="n">
-        <v>778</v>
+        <v>988.745124485888</v>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="n">
-        <v>810</v>
+        <v>990.0000000000091</v>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="n">
-        <v>890</v>
+        <v>873.3648295009857</v>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="n">
-        <v>958</v>
+        <v>750.4974349927238</v>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="n">
-        <v>938</v>
+        <v>775.141502596739</v>
       </c>
     </row>
     <row r="455">
       <c r="A455" t="n">
-        <v>886</v>
+        <v>840.7663067035855</v>
       </c>
     </row>
     <row r="456">
       <c r="A456" t="n">
-        <v>832</v>
+        <v>922.1656893778345</v>
       </c>
     </row>
     <row r="457">
       <c r="A457" t="n">
-        <v>750</v>
+        <v>936.1472023491046</v>
       </c>
     </row>
     <row r="458">
       <c r="A458" t="n">
-        <v>740</v>
+        <v>888.6438612562415</v>
       </c>
     </row>
     <row r="459">
       <c r="A459" t="n">
-        <v>784</v>
+        <v>788.9029155695653</v>
       </c>
     </row>
     <row r="460">
       <c r="A460" t="n">
-        <v>862</v>
+        <v>646.9154497969498</v>
       </c>
     </row>
     <row r="461">
       <c r="A461" t="n">
-        <v>864</v>
+        <v>620.4037948950258</v>
       </c>
     </row>
     <row r="462">
       <c r="A462" t="n">
-        <v>914</v>
+        <v>667.2968161207109</v>
       </c>
     </row>
     <row r="463">
       <c r="A463" t="n">
-        <v>896</v>
+        <v>715.6303936806125</v>
       </c>
     </row>
     <row r="464">
       <c r="A464" t="n">
-        <v>892</v>
+        <v>695.7853023624807</v>
       </c>
     </row>
     <row r="465">
       <c r="A465" t="n">
-        <v>920</v>
+        <v>764.0179135652261</v>
       </c>
     </row>
     <row r="466">
       <c r="A466" t="n">
-        <v>946</v>
+        <v>891.0819989766878</v>
       </c>
     </row>
     <row r="467">
       <c r="A467" t="n">
-        <v>940</v>
+        <v>948.9239224673724</v>
       </c>
     </row>
     <row r="468">
       <c r="A468" t="n">
-        <v>892</v>
+        <v>957.5433398856603</v>
       </c>
     </row>
     <row r="469">
       <c r="A469" t="n">
-        <v>790</v>
+        <v>938.040701472687</v>
       </c>
     </row>
     <row r="470">
       <c r="A470" t="n">
-        <v>782</v>
+        <v>831.5584234975972</v>
       </c>
     </row>
     <row r="471">
       <c r="A471" t="n">
-        <v>792</v>
+        <v>798.7477472026967</v>
       </c>
     </row>
     <row r="472">
       <c r="A472" t="n">
-        <v>884</v>
+        <v>768.2456833678657</v>
       </c>
     </row>
     <row r="473">
       <c r="A473" t="n">
-        <v>916</v>
+        <v>723.2369362133113</v>
       </c>
     </row>
     <row r="474">
       <c r="A474" t="n">
-        <v>918</v>
+        <v>716.9151075100331</v>
       </c>
     </row>
     <row r="475">
       <c r="A475" t="n">
-        <v>900</v>
+        <v>750.2559130599593</v>
       </c>
     </row>
     <row r="476">
       <c r="A476" t="n">
-        <v>812</v>
+        <v>794.7716325003285</v>
       </c>
     </row>
     <row r="477">
       <c r="A477" t="n">
-        <v>740</v>
+        <v>712.2169374925988</v>
       </c>
     </row>
     <row r="478">
       <c r="A478" t="n">
-        <v>740</v>
+        <v>781.8465428689478</v>
       </c>
     </row>
     <row r="479">
       <c r="A479" t="n">
-        <v>818</v>
+        <v>900.8448377139757</v>
       </c>
     </row>
     <row r="480">
       <c r="A480" t="n">
-        <v>916</v>
+        <v>928.4446301718958</v>
       </c>
     </row>
     <row r="481">
       <c r="A481" t="n">
-        <v>938</v>
+        <v>844.0101422179396</v>
       </c>
     </row>
     <row r="482">
       <c r="A482" t="n">
-        <v>900</v>
+        <v>733.7350800676177</v>
       </c>
     </row>
     <row r="483">
       <c r="A483" t="n">
-        <v>862</v>
+        <v>721.1439815675362</v>
       </c>
     </row>
     <row r="484">
       <c r="A484" t="n">
-        <v>764</v>
+        <v>745.5181522031467</v>
       </c>
     </row>
     <row r="485">
       <c r="A485" t="n">
-        <v>720</v>
+        <v>820.922111829816</v>
       </c>
     </row>
     <row r="486">
       <c r="A486" t="n">
-        <v>724</v>
+        <v>853.6028709983157</v>
       </c>
     </row>
     <row r="487">
       <c r="A487" t="n">
-        <v>800</v>
+        <v>814.0626447684554</v>
       </c>
     </row>
     <row r="488">
       <c r="A488" t="n">
-        <v>862</v>
+        <v>766.2577352865583</v>
       </c>
     </row>
     <row r="489">
       <c r="A489" t="n">
-        <v>812</v>
+        <v>757.1026763952773</v>
       </c>
     </row>
     <row r="490">
       <c r="A490" t="n">
-        <v>856</v>
+        <v>749.3523556731247</v>
       </c>
     </row>
     <row r="491">
       <c r="A491" t="n">
-        <v>798</v>
+        <v>787.3816493525965</v>
       </c>
     </row>
     <row r="492">
       <c r="A492" t="n">
-        <v>800</v>
+        <v>807.1770896569888</v>
       </c>
     </row>
     <row r="493">
       <c r="A493" t="n">
-        <v>994</v>
+        <v>824.227116798113</v>
       </c>
     </row>
     <row r="494">
       <c r="A494" t="n">
-        <v>974</v>
+        <v>796.2354742135176</v>
       </c>
     </row>
     <row r="495">
       <c r="A495" t="n">
-        <v>934</v>
+        <v>813.8223313232515</v>
       </c>
     </row>
     <row r="496">
       <c r="A496" t="n">
-        <v>822</v>
+        <v>785.5768525979556</v>
       </c>
     </row>
     <row r="497">
       <c r="A497" t="n">
-        <v>796</v>
+        <v>795.7388993649488</v>
       </c>
     </row>
     <row r="498">
       <c r="A498" t="n">
-        <v>790</v>
+        <v>778.9649361364468</v>
       </c>
     </row>
     <row r="499">
       <c r="A499" t="n">
-        <v>856</v>
+        <v>819.4986798673085</v>
       </c>
     </row>
     <row r="500">
       <c r="A500" t="n">
-        <v>912</v>
+        <v>813.2319617570261</v>
       </c>
     </row>
     <row r="501">
       <c r="A501" t="n">
-        <v>900</v>
+        <v>789.1004324989126</v>
       </c>
     </row>
     <row r="502">
       <c r="A502" t="n">
-        <v>870</v>
+        <v>811.6470523059434</v>
       </c>
     </row>
     <row r="503">
       <c r="A503" t="n">
-        <v>840</v>
+        <v>751.9804422531138</v>
       </c>
     </row>
     <row r="504">
       <c r="A504" t="n">
-        <v>790</v>
+        <v>778.3784184248361</v>
       </c>
     </row>
     <row r="505">
       <c r="A505" t="n">
-        <v>736</v>
+        <v>783.8629705461244</v>
       </c>
     </row>
     <row r="506">
       <c r="A506" t="n">
-        <v>770</v>
+        <v>791.4061507773908</v>
       </c>
     </row>
     <row r="507">
       <c r="A507" t="n">
-        <v>902</v>
+        <v>724.5812655199302</v>
       </c>
     </row>
     <row r="508">
       <c r="A508" t="n">
-        <v>956</v>
+        <v>802.2684539353691</v>
       </c>
     </row>
     <row r="509">
       <c r="A509" t="n">
-        <v>988</v>
+        <v>807.2466828741085</v>
       </c>
     </row>
     <row r="510">
       <c r="A510" t="n">
-        <v>942</v>
+        <v>782.0440701282791</v>
       </c>
     </row>
     <row r="511">
       <c r="A511" t="n">
-        <v>824</v>
+        <v>827.6127018079364</v>
       </c>
     </row>
     <row r="512">
       <c r="A512" t="n">
-        <v>780</v>
+        <v>795.0965394782656</v>
       </c>
     </row>
     <row r="513">
       <c r="A513" t="n">
-        <v>788</v>
+        <v>820.6675932474923</v>
       </c>
     </row>
     <row r="514">
       <c r="A514" t="n">
-        <v>878</v>
+        <v>832.640587314188</v>
       </c>
     </row>
     <row r="515">
       <c r="A515" t="n">
-        <v>892</v>
+        <v>781.9369872826201</v>
       </c>
     </row>
     <row r="516">
       <c r="A516" t="n">
-        <v>812</v>
+        <v>791.7212307728505</v>
       </c>
     </row>
     <row r="517">
       <c r="A517" t="n">
-        <v>824</v>
+        <v>836.5677984932631</v>
       </c>
     </row>
     <row r="518">
       <c r="A518" t="n">
-        <v>908</v>
+        <v>773.8100977556428</v>
       </c>
     </row>
     <row r="519">
       <c r="A519" t="n">
-        <v>960</v>
+        <v>652.2749411387281</v>
       </c>
     </row>
     <row r="520">
       <c r="A520" t="n">
-        <v>954</v>
+        <v>645.7445156324297</v>
       </c>
     </row>
     <row r="521">
       <c r="A521" t="n">
-        <v>932</v>
+        <v>680.0346527522834</v>
       </c>
     </row>
     <row r="522">
       <c r="A522" t="n">
-        <v>896</v>
+        <v>665.9886260660528</v>
       </c>
     </row>
     <row r="523">
       <c r="A523" t="n">
-        <v>870</v>
+        <v>665.9039646081624</v>
       </c>
     </row>
     <row r="524">
       <c r="A524" t="n">
-        <v>832</v>
+        <v>634.160012307234</v>
       </c>
     </row>
     <row r="525">
       <c r="A525" t="n">
-        <v>776</v>
+        <v>605.8951446394758</v>
       </c>
     </row>
     <row r="526">
       <c r="A526" t="n">
-        <v>788</v>
+        <v>655.1446453808012</v>
       </c>
     </row>
     <row r="527">
       <c r="A527" t="n">
-        <v>868</v>
+        <v>685.7414605590861</v>
       </c>
     </row>
     <row r="528">
       <c r="A528" t="n">
-        <v>764</v>
+        <v>675.933863915759</v>
       </c>
     </row>
     <row r="529">
       <c r="A529" t="n">
-        <v>700</v>
+        <v>688.9498010020816</v>
       </c>
     </row>
     <row r="530">
       <c r="A530" t="n">
-        <v>712</v>
+        <v>686.6897903522613</v>
       </c>
     </row>
     <row r="531">
       <c r="A531" t="n">
-        <v>738</v>
+        <v>713.5779250904193</v>
       </c>
     </row>
     <row r="532">
       <c r="A532" t="n">
-        <v>770</v>
+        <v>669.7660871107018</v>
       </c>
     </row>
     <row r="533">
       <c r="A533" t="n">
-        <v>880</v>
+        <v>655.5508820908926</v>
       </c>
     </row>
     <row r="534">
       <c r="A534" t="n">
-        <v>904</v>
+        <v>764.8383984586076</v>
       </c>
     </row>
     <row r="535">
       <c r="A535" t="n">
-        <v>888</v>
+        <v>795.0749327271751</v>
       </c>
     </row>
     <row r="536">
       <c r="A536" t="n">
-        <v>822</v>
+        <v>811.1094859085597</v>
       </c>
     </row>
     <row r="537">
       <c r="A537" t="n">
-        <v>728</v>
+        <v>736.2133077949125</v>
       </c>
     </row>
     <row r="538">
       <c r="A538" t="n">
-        <v>676</v>
+        <v>735.8172502938487</v>
       </c>
     </row>
     <row r="539">
       <c r="A539" t="n">
-        <v>650</v>
+        <v>721.9505378446343</v>
       </c>
     </row>
     <row r="540">
       <c r="A540" t="n">
-        <v>644</v>
+        <v>698.4962739227853</v>
       </c>
     </row>
     <row r="541">
       <c r="A541" t="n">
-        <v>668</v>
-      </c>
-    </row>
-    <row r="542">
-      <c r="A542" t="n">
-        <v>784</v>
-      </c>
-    </row>
-    <row r="543">
-      <c r="A543" t="n">
-        <v>890</v>
+        <v>721.7620573740078</v>
       </c>
     </row>
   </sheetData>

</xml_diff>